<commit_message>
Add editable chart titles, native curve styles and row-oriented RvR selection
</commit_message>
<xml_diff>
--- a/docs/rvr-excel-template.xlsx
+++ b/docs/rvr-excel-template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Single" sheetId="1" r:id="Re8564f159e704e7e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TxBF" sheetId="2" r:id="R9414240c882846a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Single" sheetId="1" r:id="Rc9b07b79e0f84b10"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TxBF" sheetId="2" r:id="R773b0245b0174c93"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -75,7 +75,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="13">
+  <x:cellXfs count="14">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -95,6 +95,9 @@
     <x:xf numFmtId="200" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="right"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -109,20 +112,15 @@
   <c:chart>
     <c:title>
       <c:tx>
-        <c:rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:r>
-              <a:rPr sz="1200">
-                <a:latin typeface="Arial"/>
-                <a:ea typeface="Arial"/>
-                <a:cs typeface="Arial"/>
-              </a:rPr>
-              <a:t>RvR throughput</a:t>
-            </a:r>
-          </a:p>
-        </c:rich>
+        <c:strRef>
+          <c:f>'Single'!$A$2</c:f>
+          <c:strCache>
+            <c:ptCount val="1"/>
+            <c:pt idx="0">
+              <c:v>RvR Throughput</c:v>
+            </c:pt>
+          </c:strCache>
+        </c:strRef>
       </c:tx>
       <c:overlay val="0"/>
       <c:txPr>
@@ -147,7 +145,15 @@
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:tx>
-            <c:v>Throughput</c:v>
+            <c:strRef>
+              <c:f>'Single'!$B$6</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Throughput (Mbps)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
           </c:tx>
           <c:spPr>
             <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
@@ -182,6 +188,7 @@
               </c:numCache>
             </c:numRef>
           </c:yVal>
+          <c:smooth val="0"/>
         </c:ser>
         <c:axId val="48650112"/>
         <c:axId val="48672768"/>
@@ -309,20 +316,15 @@
   <c:chart>
     <c:title>
       <c:tx>
-        <c:rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:r>
-              <a:rPr sz="1200">
-                <a:latin typeface="Arial"/>
-                <a:ea typeface="Arial"/>
-                <a:cs typeface="Arial"/>
-              </a:rPr>
-              <a:t>TxBF ON / OFF RvR</a:t>
-            </a:r>
-          </a:p>
-        </c:rich>
+        <c:strRef>
+          <c:f>'TxBF'!$A$2</c:f>
+          <c:strCache>
+            <c:ptCount val="1"/>
+            <c:pt idx="0">
+              <c:v>TxBF ON / OFF RvR</c:v>
+            </c:pt>
+          </c:strCache>
+        </c:strRef>
       </c:tx>
       <c:overlay val="0"/>
       <c:txPr>
@@ -347,7 +349,15 @@
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:tx>
-            <c:v>TxBF ON</c:v>
+            <c:strRef>
+              <c:f>'TxBF'!$B$6</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>TxBF ON</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
           </c:tx>
           <c:spPr>
             <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
@@ -382,12 +392,21 @@
               </c:numCache>
             </c:numRef>
           </c:yVal>
+          <c:smooth val="0"/>
         </c:ser>
         <c:ser>
           <c:idx val="1"/>
           <c:order val="1"/>
           <c:tx>
-            <c:v>TxBF OFF</c:v>
+            <c:strRef>
+              <c:f>'TxBF'!$E$6</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>TxBF OFF</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
           </c:tx>
           <c:spPr>
             <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
@@ -422,6 +441,7 @@
               </c:numCache>
             </c:numRef>
           </c:yVal>
+          <c:smooth val="0"/>
         </c:ser>
         <c:axId val="48650112"/>
         <c:axId val="48672768"/>
@@ -585,7 +605,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd4b7d7bb9d984f21"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb6c4721ac4dc4e75"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -620,7 +640,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R04afe7438e564139"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra730928877a04676"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -888,7 +908,7 @@
     </x:row>
     <x:row r="3" ht="23" customHeight="1">
       <x:c r="A3" s="3" t="str">
-        <x:v>Paste numeric dB / Mbps pairs from row 7. Up to 1,000 points per series.</x:v>
+        <x:v>Edit A2 for chart title. Paste up to 1,000 numeric X/Y pairs from row 7.</x:v>
       </x:c>
       <x:c r="B3" s="1"/>
       <x:c r="C3" s="1"/>
@@ -930,7 +950,7 @@
     </x:row>
     <x:row r="5" ht="23" customHeight="1">
       <x:c r="A5" s="3" t="str">
-        <x:v>Clear old rows before pasting. Blank = unmeasured; numeric 0 = measured zero.</x:v>
+        <x:v>Edit B6 for legend. Right-click chart to select data or format series. Blank = unmeasured.</x:v>
       </x:c>
       <x:c r="B5" s="1"/>
       <x:c r="C5" s="1"/>
@@ -949,11 +969,11 @@
       <x:c r="P5" s="1"/>
       <x:c r="Q5" s="1"/>
     </x:row>
-    <x:row r="6" ht="30" customHeight="1">
-      <x:c r="A6" s="6" t="str">
-        <x:v>Attenuation (dB)</x:v>
+    <x:row r="6" ht="42" customHeight="1">
+      <x:c r="A6" s="13" t="str">
+        <x:v>dB</x:v>
       </x:c>
-      <x:c r="B6" s="6" t="str">
+      <x:c r="B6" s="13" t="str">
         <x:v>Throughput (Mbps)</x:v>
       </x:c>
       <x:c r="C6" s="1"/>
@@ -5414,7 +5434,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5910a6d5db8d4d2c"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re78546ff74b1496d"/>
 </x:worksheet>
 </file>
 
@@ -5465,7 +5485,7 @@
     </x:row>
     <x:row r="2" ht="23" customHeight="1">
       <x:c r="A2" s="2" t="str">
-        <x:v>RvR TxBF ON / OFF</x:v>
+        <x:v>TxBF ON / OFF RvR</x:v>
       </x:c>
       <x:c r="B2" s="1"/>
       <x:c r="C2" s="1"/>
@@ -5486,7 +5506,7 @@
     </x:row>
     <x:row r="3" ht="23" customHeight="1">
       <x:c r="A3" s="3" t="str">
-        <x:v>Paste numeric dB / Mbps pairs from row 7. Up to 1,000 points per series.</x:v>
+        <x:v>Edit A2 for chart title. Paste up to 1,000 numeric X/Y pairs from row 7.</x:v>
       </x:c>
       <x:c r="B3" s="1"/>
       <x:c r="C3" s="1"/>
@@ -5528,7 +5548,7 @@
     </x:row>
     <x:row r="5" ht="23" customHeight="1">
       <x:c r="A5" s="3" t="str">
-        <x:v>ON: A/B. OFF: D/E. Clear old rows before pasting. Keep each pair together.</x:v>
+        <x:v>ON: A/B. OFF: D/E. Edit B6/E6 for legends. Right-click chart to select data or format series.</x:v>
       </x:c>
       <x:c r="B5" s="1"/>
       <x:c r="C5" s="1"/>
@@ -5547,19 +5567,19 @@
       <x:c r="P5" s="1"/>
       <x:c r="Q5" s="1"/>
     </x:row>
-    <x:row r="6" ht="30" customHeight="1">
-      <x:c r="A6" s="6" t="str">
-        <x:v>Attenuation (dB)</x:v>
+    <x:row r="6" ht="42" customHeight="1">
+      <x:c r="A6" s="13" t="str">
+        <x:v>dB</x:v>
       </x:c>
-      <x:c r="B6" s="6" t="str">
-        <x:v>TxBF ON (Mbps)</x:v>
+      <x:c r="B6" s="13" t="str">
+        <x:v>TxBF ON</x:v>
       </x:c>
       <x:c r="C6" s="1"/>
-      <x:c r="D6" s="6" t="str">
-        <x:v>Attenuation (dB)</x:v>
+      <x:c r="D6" s="13" t="str">
+        <x:v>dB</x:v>
       </x:c>
-      <x:c r="E6" s="6" t="str">
-        <x:v>TxBF OFF (Mbps)</x:v>
+      <x:c r="E6" s="13" t="str">
+        <x:v>TxBF OFF</x:v>
       </x:c>
       <x:c r="F6" s="1"/>
       <x:c r="G6" s="1"/>
@@ -11961,6 +11981,6 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8243a13e56d146d0"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2ee8134f18a14afb"/>
 </x:worksheet>
 </file>
</xml_diff>